<commit_message>
updated database added cavan and derry
</commit_message>
<xml_diff>
--- a/Database.xlsx
+++ b/Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6112e55300fcb9f7/Documents/FL_Studio/Music/Pink_Noise/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="349" documentId="8_{261B944D-3154-41C4-A810-0FE7F57DCA2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC3657BD-DF47-4D11-833A-ACEC093A1C45}"/>
+  <xr:revisionPtr revIDLastSave="360" documentId="8_{261B944D-3154-41C4-A810-0FE7F57DCA2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70DB4FBF-8777-44F1-8F1E-39878AC95DE9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DFD942CF-3A3C-44FC-9CE1-5077A113D16C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="323">
   <si>
     <t>Artist</t>
   </si>
@@ -906,6 +906,105 @@
   </si>
   <si>
     <t>https://brokenteethundergums.bandcamp.com/music</t>
+  </si>
+  <si>
+    <t>Atmospheric, Sludge, Drone</t>
+  </si>
+  <si>
+    <t>https://skellignoise.bandcamp.com</t>
+  </si>
+  <si>
+    <t>Skellig</t>
+  </si>
+  <si>
+    <t>A Farewell To Hexes</t>
+  </si>
+  <si>
+    <t>Derry</t>
+  </si>
+  <si>
+    <t>Electronic, Ambient, Drone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://adamleonard.bandcamp.com/album/rendlesham </t>
+  </si>
+  <si>
+    <t>Cool Deep Sea Box</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/cooldeepseabox/</t>
+  </si>
+  <si>
+    <t>Don't Think</t>
+  </si>
+  <si>
+    <t>Cork/Dublin</t>
+  </si>
+  <si>
+    <t>https://dont-think.bandcamp.com/</t>
+  </si>
+  <si>
+    <t>biNOMiAL</t>
+  </si>
+  <si>
+    <t>Ambient, Drone, Post-Rock</t>
+  </si>
+  <si>
+    <t>https://binomial.bandcamp.com/</t>
+  </si>
+  <si>
+    <t>Zinc.fnd</t>
+  </si>
+  <si>
+    <t>https://on.soundcloud.com/ffCuBy5AMYJQLVtGsn</t>
+  </si>
+  <si>
+    <t>Aroomabang</t>
+  </si>
+  <si>
+    <t>https://youtu.be/DRQXbDuZIgA?is=4iqFttLZBuK6PkXN</t>
+  </si>
+  <si>
+    <t>Cavan</t>
+  </si>
+  <si>
+    <t>Drone, Ambient, Techno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electronica, IDM, Braindance </t>
+  </si>
+  <si>
+    <t>Ambient, Drone, Tape-Cut Ups</t>
+  </si>
+  <si>
+    <t>https://amalgamatedwondersoftheworld.bandcamp.com/</t>
+  </si>
+  <si>
+    <t>AMALGAMATED WONDERS OF THE WORLD</t>
+  </si>
+  <si>
+    <t>Jelena Perišić</t>
+  </si>
+  <si>
+    <t>https://jelenaperisic.bandcamp.com/</t>
+  </si>
+  <si>
+    <t>Musique concrète, Minimalism, Sound art</t>
+  </si>
+  <si>
+    <t>Magnata Music</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/magnata.musick/</t>
+  </si>
+  <si>
+    <t>Drone, Noise, Pop</t>
+  </si>
+  <si>
+    <t>Solo, Electronics</t>
+  </si>
+  <si>
+    <t>Solo/Studio</t>
   </si>
 </sst>
 </file>
@@ -981,7 +1080,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -999,6 +1098,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1334,7 +1437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A5A2A8A-70C6-4D0F-949E-432942F6B4F0}">
-  <dimension ref="A1:JJ98"/>
+  <dimension ref="A1:JJ108"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" style="2" bestFit="1" customWidth="1"/>
@@ -18847,6 +18950,173 @@
       <c r="D98" s="2" t="s">
         <v>289</v>
       </c>
+      <c r="E98" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>292</v>
+      </c>
+      <c r="B99" t="s">
+        <v>75</v>
+      </c>
+      <c r="C99" t="s">
+        <v>290</v>
+      </c>
+      <c r="D99" t="s">
+        <v>291</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>293</v>
+      </c>
+      <c r="B100" t="s">
+        <v>294</v>
+      </c>
+      <c r="C100" t="s">
+        <v>295</v>
+      </c>
+      <c r="D100" t="s">
+        <v>296</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>297</v>
+      </c>
+      <c r="B101" t="s">
+        <v>56</v>
+      </c>
+      <c r="C101" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>299</v>
+      </c>
+      <c r="B102" t="s">
+        <v>300</v>
+      </c>
+      <c r="C102" t="s">
+        <v>47</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>302</v>
+      </c>
+      <c r="B103" t="s">
+        <v>36</v>
+      </c>
+      <c r="C103" t="s">
+        <v>303</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>305</v>
+      </c>
+      <c r="B104" t="s">
+        <v>56</v>
+      </c>
+      <c r="C104" t="s">
+        <v>311</v>
+      </c>
+      <c r="D104" t="s">
+        <v>306</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>307</v>
+      </c>
+      <c r="B105" t="s">
+        <v>309</v>
+      </c>
+      <c r="C105" t="s">
+        <v>310</v>
+      </c>
+      <c r="D105" t="s">
+        <v>308</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A106" s="13" t="s">
+        <v>314</v>
+      </c>
+      <c r="B106" t="s">
+        <v>36</v>
+      </c>
+      <c r="C106" t="s">
+        <v>312</v>
+      </c>
+      <c r="D106" s="14" t="s">
+        <v>313</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>315</v>
+      </c>
+      <c r="B107" t="s">
+        <v>56</v>
+      </c>
+      <c r="C107" t="s">
+        <v>317</v>
+      </c>
+      <c r="D107" t="s">
+        <v>316</v>
+      </c>
+      <c r="E107" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>318</v>
+      </c>
+      <c r="B108" t="s">
+        <v>29</v>
+      </c>
+      <c r="C108" t="s">
+        <v>320</v>
+      </c>
+      <c r="D108" t="s">
+        <v>319</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E93">
@@ -18899,6 +19169,7 @@
     <hyperlink ref="D37" r:id="rId44" xr:uid="{C4E727AC-64EB-4160-96AC-12CBDF0524FE}"/>
     <hyperlink ref="D16" r:id="rId45" xr:uid="{BEE4E429-D960-4C01-8ADA-696A4947C19F}"/>
     <hyperlink ref="A95" r:id="rId46" display="https://soundcloud.com/fionnualabloemdoran" xr:uid="{4AC40DFC-C1A9-4F16-8995-4A32EAF51800}"/>
+    <hyperlink ref="D106" r:id="rId47" xr:uid="{F239B9F6-64FF-4D37-9E43-160315944141}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed links in database
</commit_message>
<xml_diff>
--- a/Database.xlsx
+++ b/Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6112e55300fcb9f7/Documents/FL_Studio/Music/Pink_Noise/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="361" documentId="8_{261B944D-3154-41C4-A810-0FE7F57DCA2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27E1C211-6A81-4959-AB74-98978E35C4CC}"/>
+  <xr:revisionPtr revIDLastSave="367" documentId="8_{261B944D-3154-41C4-A810-0FE7F57DCA2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4D4C11D-A018-4024-9AAB-4E3222CCD6F2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DFD942CF-3A3C-44FC-9CE1-5077A113D16C}"/>
   </bookViews>
@@ -653,9 +653,6 @@
     <t>Paddy Mulcahy</t>
   </si>
   <si>
-    <t>www.paddymulcahy.com</t>
-  </si>
-  <si>
     <t>Patrick Corcoran</t>
   </si>
   <si>
@@ -830,9 +827,6 @@
     <t>Tony Monahan</t>
   </si>
   <si>
-    <t>www.tonymonahan.com</t>
-  </si>
-  <si>
     <t>Wheat Flats Press</t>
   </si>
   <si>
@@ -1022,9 +1016,6 @@
     <t>Acid House, Ambient dub, Experimental Dance</t>
   </si>
   <si>
-    <t>oorm.bandcamp.com</t>
-  </si>
-  <si>
     <t>Heironull</t>
   </si>
   <si>
@@ -1032,6 +1023,15 @@
   </si>
   <si>
     <t>https://heironull.bandcamp.com/</t>
+  </si>
+  <si>
+    <t>https://www.paddymulcahy.com/</t>
+  </si>
+  <si>
+    <t>https://www.tonymonahan.com/</t>
+  </si>
+  <si>
+    <t>https://oorm.bandcamp.com/music</t>
   </si>
 </sst>
 </file>
@@ -1107,7 +1107,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1129,6 +1129,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -12681,8 +12682,8 @@
       <c r="C67" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D67" s="8" t="s">
-        <v>205</v>
+      <c r="D67" s="15" t="s">
+        <v>329</v>
       </c>
       <c r="E67" s="4" t="s">
         <v>18</v>
@@ -12955,16 +12956,16 @@
     </row>
     <row r="68" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>56</v>
       </c>
       <c r="C68" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D68" s="10" t="s">
         <v>207</v>
-      </c>
-      <c r="D68" s="10" t="s">
-        <v>208</v>
       </c>
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
@@ -13234,16 +13235,16 @@
     </row>
     <row r="69" spans="1:270" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>56</v>
       </c>
       <c r="C69" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="D69" s="9" t="s">
         <v>210</v>
-      </c>
-      <c r="D69" s="9" t="s">
-        <v>211</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>10</v>
@@ -13516,7 +13517,7 @@
     </row>
     <row r="70" spans="1:270" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>75</v>
@@ -13525,7 +13526,7 @@
         <v>121</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E70" s="4" t="s">
         <v>18</v>
@@ -13798,16 +13799,16 @@
     </row>
     <row r="71" spans="1:270" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>43</v>
       </c>
       <c r="C71" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="D71" s="8" t="s">
         <v>215</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>216</v>
       </c>
       <c r="E71" s="4" t="s">
         <v>18</v>
@@ -14080,16 +14081,16 @@
     </row>
     <row r="72" spans="1:270" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C72" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="D72" s="8" t="s">
         <v>218</v>
-      </c>
-      <c r="D72" s="8" t="s">
-        <v>219</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>18</v>
@@ -14362,16 +14363,16 @@
     </row>
     <row r="73" spans="1:270" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B73" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="B73" s="3" t="s">
+      <c r="C73" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="C73" s="3" t="s">
+      <c r="D73" s="9" t="s">
         <v>222</v>
-      </c>
-      <c r="D73" s="9" t="s">
-        <v>223</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>10</v>
@@ -14644,7 +14645,7 @@
     </row>
     <row r="74" spans="1:270" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>56</v>
@@ -14653,7 +14654,7 @@
         <v>76</v>
       </c>
       <c r="D74" s="10" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E74" s="2"/>
       <c r="F74" s="1"/>
@@ -14924,16 +14925,16 @@
     </row>
     <row r="75" spans="1:270" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>75</v>
       </c>
       <c r="C75" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="D75" s="2" t="s">
         <v>227</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>228</v>
       </c>
       <c r="E75" s="2"/>
       <c r="F75" s="1"/>
@@ -15204,16 +15205,16 @@
     </row>
     <row r="76" spans="1:270" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>66</v>
       </c>
       <c r="C76" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="D76" s="8" t="s">
         <v>230</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>231</v>
       </c>
       <c r="E76" s="4" t="s">
         <v>18</v>
@@ -15486,16 +15487,16 @@
     </row>
     <row r="77" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B77" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C77" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>233</v>
-      </c>
-      <c r="D77" s="2" t="s">
-        <v>234</v>
       </c>
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
@@ -15765,16 +15766,16 @@
     </row>
     <row r="78" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B78" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C78" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D78" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>237</v>
       </c>
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
@@ -16044,16 +16045,16 @@
     </row>
     <row r="79" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A79" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C79" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="D79" s="8" t="s">
         <v>239</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>240</v>
       </c>
       <c r="E79" s="4" t="s">
         <v>18</v>
@@ -16326,7 +16327,7 @@
     </row>
     <row r="80" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>36</v>
@@ -16335,7 +16336,7 @@
         <v>33</v>
       </c>
       <c r="D80" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E80" s="4" t="s">
         <v>18</v>
@@ -16608,16 +16609,16 @@
     </row>
     <row r="81" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A81" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B81" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="B81" s="4" t="s">
+      <c r="C81" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="C81" s="4" t="s">
+      <c r="D81" s="8" t="s">
         <v>245</v>
-      </c>
-      <c r="D81" s="8" t="s">
-        <v>246</v>
       </c>
       <c r="E81" s="4" t="s">
         <v>18</v>
@@ -16890,16 +16891,16 @@
     </row>
     <row r="82" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B82" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C82" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="D82" s="2" t="s">
         <v>248</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>249</v>
       </c>
       <c r="F82" s="1"/>
       <c r="G82" s="1"/>
@@ -17169,7 +17170,7 @@
     </row>
     <row r="83" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
@@ -17439,16 +17440,16 @@
     </row>
     <row r="84" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>56</v>
       </c>
       <c r="C84" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="D84" s="3" t="s">
         <v>252</v>
-      </c>
-      <c r="D84" s="3" t="s">
-        <v>253</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>10</v>
@@ -17721,16 +17722,16 @@
     </row>
     <row r="85" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>75</v>
       </c>
       <c r="C85" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D85" s="10" t="s">
         <v>255</v>
-      </c>
-      <c r="D85" s="10" t="s">
-        <v>256</v>
       </c>
       <c r="F85" s="1"/>
       <c r="G85" s="1"/>
@@ -18000,16 +18001,16 @@
     </row>
     <row r="86" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>75</v>
       </c>
       <c r="C86" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="D86" s="10" t="s">
         <v>258</v>
-      </c>
-      <c r="D86" s="10" t="s">
-        <v>259</v>
       </c>
       <c r="F86" s="1"/>
       <c r="G86" s="1"/>
@@ -18279,7 +18280,7 @@
     </row>
     <row r="87" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F87" s="1"/>
       <c r="G87" s="1"/>
@@ -18549,7 +18550,7 @@
     </row>
     <row r="88" spans="1:270" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>24</v>
@@ -18558,7 +18559,7 @@
         <v>103</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E88" s="2"/>
       <c r="F88" s="1"/>
@@ -18829,7 +18830,7 @@
     </row>
     <row r="89" spans="1:270" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>56</v>
@@ -18838,7 +18839,7 @@
         <v>16</v>
       </c>
       <c r="D89" s="8" t="s">
-        <v>264</v>
+        <v>330</v>
       </c>
       <c r="E89" s="4" t="s">
         <v>18</v>
@@ -18846,14 +18847,14 @@
     </row>
     <row r="90" spans="1:270" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>75</v>
       </c>
       <c r="C90" s="5"/>
       <c r="D90" s="11" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="E90" s="5" t="s">
         <v>69</v>
@@ -18861,36 +18862,36 @@
     </row>
     <row r="91" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="92" spans="1:270" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="E92" s="2"/>
     </row>
     <row r="93" spans="1:270" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B93" s="4" t="s">
         <v>43</v>
@@ -18899,7 +18900,7 @@
         <v>200</v>
       </c>
       <c r="D93" s="8" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E93" s="4" t="s">
         <v>18</v>
@@ -18907,16 +18908,16 @@
     </row>
     <row r="94" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>18</v>
@@ -18924,13 +18925,13 @@
     </row>
     <row r="95" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A95" s="12" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C95" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>18</v>
@@ -18938,27 +18939,27 @@
     </row>
     <row r="96" spans="1:270" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="C96" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="C96" s="2" t="s">
-        <v>282</v>
-      </c>
       <c r="D96" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C97" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="B97" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>286</v>
-      </c>
       <c r="D97" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>18</v>
@@ -18966,16 +18967,16 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>18</v>
@@ -18983,16 +18984,16 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B99" t="s">
         <v>75</v>
       </c>
       <c r="C99" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D99" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>18</v>
@@ -19000,16 +19001,16 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>291</v>
+      </c>
+      <c r="B100" t="s">
+        <v>292</v>
+      </c>
+      <c r="C100" t="s">
         <v>293</v>
       </c>
-      <c r="B100" t="s">
+      <c r="D100" t="s">
         <v>294</v>
-      </c>
-      <c r="C100" t="s">
-        <v>295</v>
-      </c>
-      <c r="D100" t="s">
-        <v>296</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>18</v>
@@ -19017,7 +19018,7 @@
     </row>
     <row r="101" spans="1:5" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B101" t="s">
         <v>56</v>
@@ -19026,38 +19027,38 @@
         <v>76</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B102" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C102" t="s">
         <v>47</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B103" t="s">
         <v>36</v>
       </c>
       <c r="C103" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>18</v>
@@ -19065,16 +19066,16 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="B104" t="s">
         <v>56</v>
       </c>
       <c r="C104" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D104" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="E104" s="2" t="s">
         <v>18</v>
@@ -19082,16 +19083,16 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
+        <v>305</v>
+      </c>
+      <c r="B105" t="s">
         <v>307</v>
       </c>
-      <c r="B105" t="s">
-        <v>309</v>
-      </c>
       <c r="C105" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D105" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>18</v>
@@ -19099,33 +19100,33 @@
     </row>
     <row r="106" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="13" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B106" t="s">
         <v>36</v>
       </c>
       <c r="C106" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D106" s="14" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B107" t="s">
         <v>56</v>
       </c>
       <c r="C107" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D107" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="E107" s="2" t="s">
         <v>18</v>
@@ -19133,58 +19134,58 @@
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="B108" t="s">
         <v>29</v>
       </c>
       <c r="C108" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D108" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>321</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="C109" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="B109" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="C109" s="2" t="s">
-        <v>325</v>
-      </c>
       <c r="D109" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>75</v>
       </c>
       <c r="C110" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="D110" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B111" t="s">
         <v>36</v>
       </c>
       <c r="C111" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="D111" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -19192,53 +19193,52 @@
     <sortCondition ref="A2:A93"/>
   </sortState>
   <hyperlinks>
-    <hyperlink ref="D67" r:id="rId1" xr:uid="{CCB55DC0-18EB-4D96-BE27-A4F9FDAF49A3}"/>
-    <hyperlink ref="D89" r:id="rId2" xr:uid="{5A37D94E-0373-4CA0-B757-1D732381263F}"/>
-    <hyperlink ref="D68" r:id="rId3" xr:uid="{5C11DED6-BB10-449D-9A82-6C2A6D838A11}"/>
-    <hyperlink ref="D51" r:id="rId4" xr:uid="{6E53BC9F-2191-4B50-BB4B-344BF739C495}"/>
-    <hyperlink ref="D54" r:id="rId5" xr:uid="{0162C932-5F31-4C42-AD7B-A877EF27CFBD}"/>
-    <hyperlink ref="D40" r:id="rId6" xr:uid="{06BDB73F-49D5-4446-AEF7-4BAF66CA62EC}"/>
-    <hyperlink ref="D47" r:id="rId7" xr:uid="{6A597E2D-F977-4F6A-B5FE-92B378EE8AE4}"/>
-    <hyperlink ref="D21" r:id="rId8" xr:uid="{7B0B3B19-2577-4516-9564-6626CFB0AE88}"/>
-    <hyperlink ref="D59" r:id="rId9" xr:uid="{4A0A1568-A229-43D7-88C1-C2C8F704672A}"/>
-    <hyperlink ref="D70" r:id="rId10" xr:uid="{75B784A1-60FB-487A-96AC-3666C9B126EF}"/>
-    <hyperlink ref="D23" r:id="rId11" xr:uid="{A822FF5E-B570-4882-88AC-0697ED866137}"/>
-    <hyperlink ref="D64" r:id="rId12" xr:uid="{EFC1DE87-6580-436F-AB42-96A494AF275B}"/>
-    <hyperlink ref="D81" r:id="rId13" xr:uid="{A89D8F21-645A-435D-91F6-08041B8ACE6A}"/>
-    <hyperlink ref="D74" r:id="rId14" xr:uid="{4B379C73-CE24-4C05-B083-C73BCF5BE915}"/>
-    <hyperlink ref="D31" r:id="rId15" xr:uid="{34486018-4237-4C25-B096-58C199032A86}"/>
-    <hyperlink ref="D12" r:id="rId16" xr:uid="{C512F059-B0DA-4081-9219-B1171DF277F9}"/>
-    <hyperlink ref="D69" r:id="rId17" xr:uid="{ED2B95DE-8D5D-453D-88A5-08A3574133D9}"/>
-    <hyperlink ref="D86" r:id="rId18" xr:uid="{1FC48E13-3B45-4841-A63F-814420BAB3D9}"/>
-    <hyperlink ref="D14" r:id="rId19" xr:uid="{EAB70F73-F452-464D-8494-D8313411AC87}"/>
-    <hyperlink ref="D85" r:id="rId20" xr:uid="{D1E15C48-D09F-42E5-A397-BAA1B22A37EA}"/>
-    <hyperlink ref="D80" r:id="rId21" xr:uid="{F4974A41-060A-4F82-AB87-57C0FA7149F5}"/>
-    <hyperlink ref="D41" r:id="rId22" xr:uid="{680916C5-961D-4B1B-956B-F2B7F8A44EEE}"/>
-    <hyperlink ref="D35" r:id="rId23" xr:uid="{84E1707F-C979-4005-8083-1BCBF25F7C5B}"/>
-    <hyperlink ref="D30" r:id="rId24" xr:uid="{F5C7EB7E-9B78-46B8-8481-E5155FE5C82D}"/>
-    <hyperlink ref="D52" r:id="rId25" xr:uid="{BA819352-086D-405D-90E6-7118250841A3}"/>
-    <hyperlink ref="D76" r:id="rId26" xr:uid="{A7772422-2115-424E-A67F-3C57D35B7A5B}"/>
-    <hyperlink ref="D33" r:id="rId27" xr:uid="{114322D1-C7E8-4BBD-B19B-06F2595FD07B}"/>
-    <hyperlink ref="D20" r:id="rId28" xr:uid="{C886F560-887D-488F-810A-D3B1A6E3CC46}"/>
-    <hyperlink ref="D11" r:id="rId29" xr:uid="{0D344D31-67B0-48C4-8794-69011131B5B4}"/>
-    <hyperlink ref="D90" r:id="rId30" xr:uid="{EB3A9261-28FD-4F85-BEE3-D9624F0E05C9}"/>
-    <hyperlink ref="D61" r:id="rId31" xr:uid="{7EE8A41C-7770-41A4-B094-E599F03F0A14}"/>
-    <hyperlink ref="D73" r:id="rId32" xr:uid="{C2F689C9-0C1C-4060-91DE-41331706A150}"/>
-    <hyperlink ref="D93" r:id="rId33" xr:uid="{0D757BC2-FAD9-42C0-A845-FF834C07B19E}"/>
-    <hyperlink ref="D27" r:id="rId34" xr:uid="{DBA900D4-6F72-4123-A5CD-3059EDAB6302}"/>
-    <hyperlink ref="D34" r:id="rId35" xr:uid="{6BB702BC-593E-4A75-8D44-007EAC685735}"/>
-    <hyperlink ref="D36" r:id="rId36" xr:uid="{05EEFFE4-91F6-4889-B834-45F3E447E5AC}"/>
-    <hyperlink ref="D71" r:id="rId37" xr:uid="{88C26B57-A3D3-4E8E-833B-F2CDA9A762BF}"/>
-    <hyperlink ref="D29" r:id="rId38" xr:uid="{630E7085-9136-46D5-A597-896B59EBCDD2}"/>
-    <hyperlink ref="D63" r:id="rId39" xr:uid="{FB21CDE8-97FB-44F7-9340-A318935538E8}"/>
-    <hyperlink ref="D7" r:id="rId40" xr:uid="{D2E6BEFE-81EA-4E58-B4C0-EA2C73E9EF41}"/>
-    <hyperlink ref="D65" r:id="rId41" xr:uid="{E8BA0715-9825-4A8A-8DF4-20A48B1FEAD5}"/>
-    <hyperlink ref="D79" r:id="rId42" xr:uid="{4C4515D2-16F4-4812-A73B-B58944B89010}"/>
-    <hyperlink ref="D66" r:id="rId43" xr:uid="{ED5B7EF3-7CDD-4156-999C-01977C237F2B}"/>
-    <hyperlink ref="D37" r:id="rId44" xr:uid="{C4E727AC-64EB-4160-96AC-12CBDF0524FE}"/>
-    <hyperlink ref="D16" r:id="rId45" xr:uid="{BEE4E429-D960-4C01-8ADA-696A4947C19F}"/>
-    <hyperlink ref="A95" r:id="rId46" display="https://soundcloud.com/fionnualabloemdoran" xr:uid="{4AC40DFC-C1A9-4F16-8995-4A32EAF51800}"/>
-    <hyperlink ref="D106" r:id="rId47" xr:uid="{F239B9F6-64FF-4D37-9E43-160315944141}"/>
+    <hyperlink ref="D68" r:id="rId1" xr:uid="{5C11DED6-BB10-449D-9A82-6C2A6D838A11}"/>
+    <hyperlink ref="D51" r:id="rId2" xr:uid="{6E53BC9F-2191-4B50-BB4B-344BF739C495}"/>
+    <hyperlink ref="D54" r:id="rId3" xr:uid="{0162C932-5F31-4C42-AD7B-A877EF27CFBD}"/>
+    <hyperlink ref="D40" r:id="rId4" xr:uid="{06BDB73F-49D5-4446-AEF7-4BAF66CA62EC}"/>
+    <hyperlink ref="D47" r:id="rId5" xr:uid="{6A597E2D-F977-4F6A-B5FE-92B378EE8AE4}"/>
+    <hyperlink ref="D21" r:id="rId6" xr:uid="{7B0B3B19-2577-4516-9564-6626CFB0AE88}"/>
+    <hyperlink ref="D59" r:id="rId7" xr:uid="{4A0A1568-A229-43D7-88C1-C2C8F704672A}"/>
+    <hyperlink ref="D70" r:id="rId8" xr:uid="{75B784A1-60FB-487A-96AC-3666C9B126EF}"/>
+    <hyperlink ref="D23" r:id="rId9" xr:uid="{A822FF5E-B570-4882-88AC-0697ED866137}"/>
+    <hyperlink ref="D64" r:id="rId10" xr:uid="{EFC1DE87-6580-436F-AB42-96A494AF275B}"/>
+    <hyperlink ref="D81" r:id="rId11" xr:uid="{A89D8F21-645A-435D-91F6-08041B8ACE6A}"/>
+    <hyperlink ref="D74" r:id="rId12" xr:uid="{4B379C73-CE24-4C05-B083-C73BCF5BE915}"/>
+    <hyperlink ref="D31" r:id="rId13" xr:uid="{34486018-4237-4C25-B096-58C199032A86}"/>
+    <hyperlink ref="D12" r:id="rId14" xr:uid="{C512F059-B0DA-4081-9219-B1171DF277F9}"/>
+    <hyperlink ref="D69" r:id="rId15" xr:uid="{ED2B95DE-8D5D-453D-88A5-08A3574133D9}"/>
+    <hyperlink ref="D86" r:id="rId16" xr:uid="{1FC48E13-3B45-4841-A63F-814420BAB3D9}"/>
+    <hyperlink ref="D14" r:id="rId17" xr:uid="{EAB70F73-F452-464D-8494-D8313411AC87}"/>
+    <hyperlink ref="D85" r:id="rId18" xr:uid="{D1E15C48-D09F-42E5-A397-BAA1B22A37EA}"/>
+    <hyperlink ref="D80" r:id="rId19" xr:uid="{F4974A41-060A-4F82-AB87-57C0FA7149F5}"/>
+    <hyperlink ref="D41" r:id="rId20" xr:uid="{680916C5-961D-4B1B-956B-F2B7F8A44EEE}"/>
+    <hyperlink ref="D35" r:id="rId21" xr:uid="{84E1707F-C979-4005-8083-1BCBF25F7C5B}"/>
+    <hyperlink ref="D30" r:id="rId22" xr:uid="{F5C7EB7E-9B78-46B8-8481-E5155FE5C82D}"/>
+    <hyperlink ref="D52" r:id="rId23" xr:uid="{BA819352-086D-405D-90E6-7118250841A3}"/>
+    <hyperlink ref="D76" r:id="rId24" xr:uid="{A7772422-2115-424E-A67F-3C57D35B7A5B}"/>
+    <hyperlink ref="D33" r:id="rId25" xr:uid="{114322D1-C7E8-4BBD-B19B-06F2595FD07B}"/>
+    <hyperlink ref="D20" r:id="rId26" xr:uid="{C886F560-887D-488F-810A-D3B1A6E3CC46}"/>
+    <hyperlink ref="D11" r:id="rId27" xr:uid="{0D344D31-67B0-48C4-8794-69011131B5B4}"/>
+    <hyperlink ref="D90" r:id="rId28" xr:uid="{EB3A9261-28FD-4F85-BEE3-D9624F0E05C9}"/>
+    <hyperlink ref="D61" r:id="rId29" xr:uid="{7EE8A41C-7770-41A4-B094-E599F03F0A14}"/>
+    <hyperlink ref="D73" r:id="rId30" xr:uid="{C2F689C9-0C1C-4060-91DE-41331706A150}"/>
+    <hyperlink ref="D93" r:id="rId31" xr:uid="{0D757BC2-FAD9-42C0-A845-FF834C07B19E}"/>
+    <hyperlink ref="D27" r:id="rId32" xr:uid="{DBA900D4-6F72-4123-A5CD-3059EDAB6302}"/>
+    <hyperlink ref="D34" r:id="rId33" xr:uid="{6BB702BC-593E-4A75-8D44-007EAC685735}"/>
+    <hyperlink ref="D36" r:id="rId34" xr:uid="{05EEFFE4-91F6-4889-B834-45F3E447E5AC}"/>
+    <hyperlink ref="D71" r:id="rId35" xr:uid="{88C26B57-A3D3-4E8E-833B-F2CDA9A762BF}"/>
+    <hyperlink ref="D29" r:id="rId36" xr:uid="{630E7085-9136-46D5-A597-896B59EBCDD2}"/>
+    <hyperlink ref="D63" r:id="rId37" xr:uid="{FB21CDE8-97FB-44F7-9340-A318935538E8}"/>
+    <hyperlink ref="D7" r:id="rId38" xr:uid="{D2E6BEFE-81EA-4E58-B4C0-EA2C73E9EF41}"/>
+    <hyperlink ref="D65" r:id="rId39" xr:uid="{E8BA0715-9825-4A8A-8DF4-20A48B1FEAD5}"/>
+    <hyperlink ref="D79" r:id="rId40" xr:uid="{4C4515D2-16F4-4812-A73B-B58944B89010}"/>
+    <hyperlink ref="D66" r:id="rId41" xr:uid="{ED5B7EF3-7CDD-4156-999C-01977C237F2B}"/>
+    <hyperlink ref="D37" r:id="rId42" xr:uid="{C4E727AC-64EB-4160-96AC-12CBDF0524FE}"/>
+    <hyperlink ref="D16" r:id="rId43" xr:uid="{BEE4E429-D960-4C01-8ADA-696A4947C19F}"/>
+    <hyperlink ref="A95" r:id="rId44" display="https://soundcloud.com/fionnualabloemdoran" xr:uid="{4AC40DFC-C1A9-4F16-8995-4A32EAF51800}"/>
+    <hyperlink ref="D106" r:id="rId45" xr:uid="{F239B9F6-64FF-4D37-9E43-160315944141}"/>
+    <hyperlink ref="D67" r:id="rId46" xr:uid="{943BE3D1-C663-4154-9464-7AB2B0B1B866}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>